<commit_message>
QR agregado y mejoras hechas
</commit_message>
<xml_diff>
--- a/asistencia.xlsx
+++ b/asistencia.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="760" yWindow="760" windowWidth="14400" windowHeight="7270" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" state="visible" r:id="rId1"/>
@@ -390,11 +390,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col width="15.90625" customWidth="1" min="1" max="1"/>
     <col width="18.81640625" customWidth="1" min="2" max="2"/>
+    <col width="32.26953125" customWidth="1" min="3" max="3"/>
+    <col width="20.453125" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -415,12 +417,12 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>12:36:22</t>
+          <t>11:36:24</t>
         </is>
       </c>
     </row>
@@ -437,17 +439,17 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>optativa</t>
+          <t>sistemas III</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>14:13:44</t>
+          <t>11:36:59</t>
         </is>
       </c>
     </row>
@@ -464,17 +466,71 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>sistemas</t>
+          <t>sistemas II</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>14:14:06</t>
+          <t>11:37:21</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Santiago Villalba</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>202120070011</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>optativa</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>11:45:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Santiago Hernández</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>20212007090</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Optativa</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>11:49:41</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Preparar proyecto para despliegue
</commit_message>
<xml_diff>
--- a/asistencia.xlsx
+++ b/asistencia.xlsx
@@ -16,7 +16,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -24,16 +24,49 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF2563EB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.5999938962981048"/>
+        <bgColor theme="4" tint="0.5999938962981048"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.7999816888943144"/>
+        <bgColor theme="4" tint="0.7999816888943144"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002563EB"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -41,12 +74,77 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="0"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thick">
+        <color theme="0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0"/>
+      </left>
+      <right/>
+      <top style="thick">
+        <color theme="0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -121,6 +219,20 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TablaAsistencia" displayName="TablaAsistencia" ref="A1:E5" headerRowCount="1">
+  <autoFilter ref="A1:E4"/>
+  <tableColumns count="5">
+    <tableColumn id="1" name="Kevin Santiago Guerrero Barragan"/>
+    <tableColumn id="2" name="202120070010"/>
+    <tableColumn id="3" name="sistemas basicos"/>
+    <tableColumn id="4" name="fecha"/>
+    <tableColumn id="5" name="hora"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -393,107 +505,108 @@
   <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
-    <col width="15.90625" customWidth="1" min="1" max="1"/>
-    <col width="18.81640625" customWidth="1" min="2" max="2"/>
-    <col width="32.26953125" customWidth="1" min="3" max="3"/>
-    <col width="20.453125" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="15" customHeight="1" thickBot="1">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>Kevin Santiago Guerrero Barragan</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="8" t="inlineStr">
         <is>
           <t>202120070010</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>optativa</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
+      <c r="C1" s="8" t="inlineStr">
+        <is>
+          <t>sistemas basicos</t>
+        </is>
+      </c>
+      <c r="D1" s="8" t="inlineStr">
+        <is>
+          <t>fecha</t>
+        </is>
+      </c>
+      <c r="E1" s="8" t="inlineStr">
+        <is>
+          <t>hora</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="15" customHeight="1" thickTop="1">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Santiago Villalba</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>202120070010</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>sistemas</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
         <is>
           <t>2026-05-24</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>11:36:24</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Kevin Santiago Guerrero Barragan</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>202120070010</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>sistemas III</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2026-05-24</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>11:36:59</t>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>13:04:54</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>Kevin Santiago Guerrero Barragan</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="1" t="inlineStr">
         <is>
           <t>202120070010</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="1" t="inlineStr">
         <is>
           <t>sistemas II</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="1" t="inlineStr">
         <is>
           <t>2026-05-24</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>11:37:21</t>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>13:04:59</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Santiago Villalba</t>
+          <t>Kevin Santiago Guerrero Barragan</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>202120070011</t>
+          <t>202120070010</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>optativa</t>
+          <t>sistemas III</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -503,24 +616,24 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>11:45:07</t>
+          <t>13:08:30</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Santiago Hernández</t>
+          <t>Santiago Villalba</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>20212007090</t>
+          <t>202120070011</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Optativa</t>
+          <t>optativa II</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -530,11 +643,14 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>11:49:41</t>
+          <t>13:08:48</t>
         </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>